<commit_message>
Correção de Falhas de finais
</commit_message>
<xml_diff>
--- a/data/jogo.xlsx
+++ b/data/jogo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmace\Documents\GitHub\PontoSemVolta\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aysla\OneDrive\Documentos\GitHub\PontoSemVolta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94313DB7-82BB-4A2C-ADFA-466994BBEA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B129EC20-CCD3-4A0C-93E6-B64E98318E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -929,16 +929,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y76"/>
-  <sheetFormatPr defaultColWidth="41" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="41" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.33203125" customWidth="1"/>
-    <col min="2" max="2" width="20.5546875" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="6.36328125" customWidth="1"/>
+    <col min="2" max="2" width="20.54296875" customWidth="1"/>
+    <col min="3" max="3" width="14.6328125" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="6" max="24" width="12.6640625" customWidth="1"/>
+    <col min="6" max="24" width="12.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1012,7 +1012,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1509,7 +1509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2219,7 +2219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2290,7 +2290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2716,7 +2716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2932,7 +2932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3003,7 +3003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3074,7 +3074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3642,7 +3642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3784,7 +3784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3806,6 +3806,9 @@
       <c r="H41">
         <v>-60</v>
       </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
       <c r="J41">
         <v>40</v>
       </c>
@@ -3852,7 +3855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -3923,7 +3926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -3994,7 +3997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4065,7 +4068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4136,7 +4139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4207,7 +4210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4278,7 +4281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4349,7 +4352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4420,7 +4423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4491,7 +4494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4562,7 +4565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4633,7 +4636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4704,7 +4707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4775,7 +4778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4846,7 +4849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
@@ -4917,7 +4920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
@@ -4988,7 +4991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
@@ -5059,7 +5062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
@@ -5130,7 +5133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -5201,7 +5204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
@@ -5272,7 +5275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
@@ -5343,7 +5346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
@@ -5414,7 +5417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
@@ -5485,7 +5488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
@@ -5556,7 +5559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
@@ -5627,7 +5630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
@@ -5698,7 +5701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
@@ -5769,7 +5772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
@@ -5840,7 +5843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
@@ -5911,7 +5914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
@@ -5982,7 +5985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
@@ -6053,7 +6056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
@@ -6124,7 +6127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
@@ -6195,7 +6198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
@@ -6266,7 +6269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>

</xml_diff>